<commit_message>
Add Presidents Cup (Jul 11-12) results
Wire "Presidents Cup" sheet to config; flighted (5 flights, top 5 per
flight from 300/240/180/120/60). 26 players scored, 50 got participation.
New overall leader: William Harnett (1070).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryan\Projects\MGA_Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30EE6F89-C749-4F07-945D-814DC2DCBA09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6512EFBF-2458-4121-B743-ACD5065BE993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50460" yWindow="1140" windowWidth="38700" windowHeight="15225" xr2:uid="{7A62B4D0-B0BC-4A36-AEF3-D444F4B3BF77}"/>
+    <workbookView xWindow="-51720" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="7" xr2:uid="{7A62B4D0-B0BC-4A36-AEF3-D444F4B3BF77}"/>
   </bookViews>
   <sheets>
     <sheet name="Member-Member 2025" sheetId="4" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Quota" sheetId="5" r:id="rId5"/>
     <sheet name="The Gerald" sheetId="6" r:id="rId6"/>
     <sheet name="Member-Member 2026" sheetId="7" r:id="rId7"/>
+    <sheet name="Presidents Cup" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="292">
   <si>
     <t>Flight 1</t>
   </si>
@@ -879,13 +880,52 @@
   </si>
   <si>
     <t>Bolen, Trey + Mueller, Shawn</t>
+  </si>
+  <si>
+    <t>Today</t>
+  </si>
+  <si>
+    <t>Fagan, Eric</t>
+  </si>
+  <si>
+    <t>Jones, Kenny</t>
+  </si>
+  <si>
+    <t>Perez, Zach</t>
+  </si>
+  <si>
+    <t>Maness, Will</t>
+  </si>
+  <si>
+    <t>Moser, Sean</t>
+  </si>
+  <si>
+    <t>Bruegel, Michael</t>
+  </si>
+  <si>
+    <t>Byrns, Ray</t>
+  </si>
+  <si>
+    <t>Bolen, Trey</t>
+  </si>
+  <si>
+    <t>Larkin, Tripp</t>
+  </si>
+  <si>
+    <t>Robertson, David</t>
+  </si>
+  <si>
+    <t>Quarles, Aaron</t>
+  </si>
+  <si>
+    <t>Schreiber, David</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -945,6 +985,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Font Awesome 6 Free"/>
     </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Font Awesome 6 Free"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -972,7 +1018,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1078,12 +1124,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD3DADE"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD3DADE"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1119,23 +1176,8 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1152,6 +1194,18 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1164,8 +1218,41 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1909,26 +1996,26 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17" customHeight="1" thickBot="1">
       <c r="A1" s="8"/>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="22"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -1936,13 +2023,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" thickBot="1">
-      <c r="A3" s="23"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="18"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="22"/>
       <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="16"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="3" t="s">
         <v>4</v>
       </c>
@@ -2119,26 +2206,26 @@
     </row>
     <row r="14" spans="1:6" ht="17" thickBot="1">
       <c r="A14" s="8"/>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="21"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="22"/>
-      <c r="B15" s="15" t="s">
+      <c r="A15" s="17"/>
+      <c r="B15" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -2146,13 +2233,13 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" thickBot="1">
-      <c r="A16" s="23"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="18"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="22"/>
       <c r="D16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="20"/>
       <c r="F16" s="3" t="s">
         <v>4</v>
       </c>
@@ -2329,26 +2416,26 @@
     </row>
     <row r="27" spans="1:6" ht="17" thickBot="1">
       <c r="A27" s="8"/>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="21"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="16"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="22"/>
-      <c r="B28" s="15" t="s">
+      <c r="A28" s="17"/>
+      <c r="B28" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F28" s="2" t="s">
@@ -2356,13 +2443,13 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="15" thickBot="1">
-      <c r="A29" s="23"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="18"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="22"/>
       <c r="D29" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="16"/>
+      <c r="E29" s="20"/>
       <c r="F29" s="3" t="s">
         <v>4</v>
       </c>
@@ -2539,26 +2626,26 @@
     </row>
     <row r="40" spans="1:6" ht="17" thickBot="1">
       <c r="A40" s="8"/>
-      <c r="B40" s="19" t="s">
+      <c r="B40" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="21"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="16"/>
     </row>
     <row r="41" spans="1:6">
-      <c r="A41" s="22"/>
-      <c r="B41" s="15" t="s">
+      <c r="A41" s="17"/>
+      <c r="B41" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="C41" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E41" s="15" t="s">
+      <c r="E41" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F41" s="2" t="s">
@@ -2566,13 +2653,13 @@
       </c>
     </row>
     <row r="42" spans="1:6" ht="15" thickBot="1">
-      <c r="A42" s="23"/>
-      <c r="B42" s="16"/>
-      <c r="C42" s="18"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="22"/>
       <c r="D42" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E42" s="16"/>
+      <c r="E42" s="20"/>
       <c r="F42" s="3" t="s">
         <v>4</v>
       </c>
@@ -2723,11 +2810,11 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="E28:E29"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B15:B16"/>
@@ -2738,11 +2825,11 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="E41:E42"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?utf8=%E2%9C%93&amp;shared=false&amp;no_header=&amp;show_tv_button=&amp;round=1560524" xr:uid="{2DEC3451-4FA2-4305-B881-362B70C975D8}"/>
@@ -2794,16 +2881,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="19" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -2812,12 +2899,12 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="15" thickBot="1">
-      <c r="A2" s="16"/>
-      <c r="B2" s="18"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="22"/>
       <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="16"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
@@ -3130,26 +3217,26 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17" customHeight="1" thickBot="1">
       <c r="A1" s="8"/>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="22"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -3157,13 +3244,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" thickBot="1">
-      <c r="A3" s="23"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="18"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="22"/>
       <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="16"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="3" t="s">
         <v>4</v>
       </c>
@@ -3340,26 +3427,26 @@
     </row>
     <row r="14" spans="1:6" ht="17" thickBot="1">
       <c r="A14" s="8"/>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="21"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="16"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="22"/>
-      <c r="B15" s="15" t="s">
+      <c r="A15" s="17"/>
+      <c r="B15" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -3367,13 +3454,13 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" thickBot="1">
-      <c r="A16" s="23"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="18"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="22"/>
       <c r="D16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="16"/>
+      <c r="E16" s="20"/>
       <c r="F16" s="3" t="s">
         <v>4</v>
       </c>
@@ -3532,26 +3619,26 @@
     </row>
     <row r="26" spans="1:6" ht="17" thickBot="1">
       <c r="A26" s="8"/>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="21"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="16"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="22"/>
-      <c r="B27" s="15" t="s">
+      <c r="A27" s="17"/>
+      <c r="B27" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="E27" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F27" s="2" t="s">
@@ -3559,13 +3646,13 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" thickBot="1">
-      <c r="A28" s="23"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="18"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="22"/>
       <c r="D28" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="16"/>
+      <c r="E28" s="20"/>
       <c r="F28" s="3" t="s">
         <v>4</v>
       </c>
@@ -3724,26 +3811,26 @@
     </row>
     <row r="38" spans="1:6" ht="17" thickBot="1">
       <c r="A38" s="8"/>
-      <c r="B38" s="19" t="s">
+      <c r="B38" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="21"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="16"/>
     </row>
     <row r="39" spans="1:6">
-      <c r="A39" s="22"/>
-      <c r="B39" s="15" t="s">
+      <c r="A39" s="17"/>
+      <c r="B39" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C39" s="17" t="s">
+      <c r="C39" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E39" s="15" t="s">
+      <c r="E39" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F39" s="2" t="s">
@@ -3751,13 +3838,13 @@
       </c>
     </row>
     <row r="40" spans="1:6" ht="15" thickBot="1">
-      <c r="A40" s="23"/>
-      <c r="B40" s="16"/>
-      <c r="C40" s="18"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="22"/>
       <c r="D40" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E40" s="16"/>
+      <c r="E40" s="20"/>
       <c r="F40" s="3" t="s">
         <v>4</v>
       </c>
@@ -3916,26 +4003,26 @@
     </row>
     <row r="50" spans="1:6" ht="17" thickBot="1">
       <c r="A50" s="8"/>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="20"/>
-      <c r="F50" s="21"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="16"/>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="22"/>
-      <c r="B51" s="15" t="s">
+      <c r="A51" s="17"/>
+      <c r="B51" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C51" s="17" t="s">
+      <c r="C51" s="21" t="s">
         <v>2</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E51" s="15" t="s">
+      <c r="E51" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F51" s="2" t="s">
@@ -3943,13 +4030,13 @@
       </c>
     </row>
     <row r="52" spans="1:6" ht="15" thickBot="1">
-      <c r="A52" s="23"/>
-      <c r="B52" s="16"/>
-      <c r="C52" s="18"/>
+      <c r="A52" s="18"/>
+      <c r="B52" s="20"/>
+      <c r="C52" s="22"/>
       <c r="D52" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E52" s="16"/>
+      <c r="E52" s="20"/>
       <c r="F52" s="3" t="s">
         <v>4</v>
       </c>
@@ -4100,6 +4187,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="A51:A52"/>
     <mergeCell ref="B51:B52"/>
     <mergeCell ref="C51:C52"/>
@@ -4116,15 +4212,6 @@
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="E15:E16"/>
     <mergeCell ref="B26:F26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B14:F14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?utf8=%E2%9C%93&amp;shared=false&amp;no_header=&amp;show_tv_button=&amp;round=1572854" xr:uid="{6DCC4AEF-9CD1-4F4E-A929-82302C2E4EDC}"/>
@@ -4179,29 +4266,29 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:8" ht="17" thickBot="1">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="21"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="16"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="26"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="25"/>
+      <c r="B2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="19" t="s">
         <v>163</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -4213,11 +4300,11 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" ht="18.5" thickBot="1">
-      <c r="A3" s="27"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
+      <c r="A3" s="26"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="3" t="s">
         <v>164</v>
       </c>
@@ -4436,28 +4523,28 @@
     </row>
     <row r="14" spans="1:8" ht="17" thickBot="1">
       <c r="A14" s="11"/>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="21"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="16"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="26"/>
-      <c r="B15" s="15" t="s">
+      <c r="A15" s="25"/>
+      <c r="B15" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="19" t="s">
         <v>163</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -4469,11 +4556,11 @@
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="1:8" ht="18.5" thickBot="1">
-      <c r="A16" s="27"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
       <c r="F16" s="3" t="s">
         <v>164</v>
       </c>
@@ -4714,28 +4801,28 @@
     </row>
     <row r="28" spans="1:8" ht="17" thickBot="1">
       <c r="A28" s="11"/>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="21"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="16"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="26"/>
-      <c r="B29" s="15" t="s">
+      <c r="A29" s="25"/>
+      <c r="B29" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="E29" s="19" t="s">
         <v>163</v>
       </c>
       <c r="F29" s="2" t="s">
@@ -4747,11 +4834,11 @@
       <c r="H29" s="1"/>
     </row>
     <row r="30" spans="1:8" ht="18.5" thickBot="1">
-      <c r="A30" s="27"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
+      <c r="A30" s="26"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
       <c r="F30" s="3" t="s">
         <v>164</v>
       </c>
@@ -4970,28 +5057,28 @@
     </row>
     <row r="41" spans="1:8" ht="17" thickBot="1">
       <c r="A41" s="11"/>
-      <c r="B41" s="19" t="s">
+      <c r="B41" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="20"/>
-      <c r="H41" s="21"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="16"/>
     </row>
     <row r="42" spans="1:8">
-      <c r="A42" s="26"/>
-      <c r="B42" s="15" t="s">
+      <c r="A42" s="25"/>
+      <c r="B42" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C42" s="17" t="s">
+      <c r="C42" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E42" s="15" t="s">
+      <c r="E42" s="19" t="s">
         <v>163</v>
       </c>
       <c r="F42" s="2" t="s">
@@ -5003,11 +5090,11 @@
       <c r="H42" s="1"/>
     </row>
     <row r="43" spans="1:8" ht="18.5" thickBot="1">
-      <c r="A43" s="27"/>
-      <c r="B43" s="16"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
+      <c r="A43" s="26"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
       <c r="F43" s="3" t="s">
         <v>164</v>
       </c>
@@ -5226,28 +5313,28 @@
     </row>
     <row r="54" spans="1:8" ht="17" thickBot="1">
       <c r="A54" s="11"/>
-      <c r="B54" s="19" t="s">
+      <c r="B54" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="20"/>
-      <c r="H54" s="21"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="16"/>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="26"/>
-      <c r="B55" s="15" t="s">
+      <c r="A55" s="25"/>
+      <c r="B55" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C55" s="17" t="s">
+      <c r="C55" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D55" s="15" t="s">
+      <c r="D55" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E55" s="15" t="s">
+      <c r="E55" s="19" t="s">
         <v>163</v>
       </c>
       <c r="F55" s="2" t="s">
@@ -5259,11 +5346,11 @@
       <c r="H55" s="1"/>
     </row>
     <row r="56" spans="1:8" ht="18.5" thickBot="1">
-      <c r="A56" s="27"/>
-      <c r="B56" s="16"/>
-      <c r="C56" s="18"/>
-      <c r="D56" s="16"/>
-      <c r="E56" s="16"/>
+      <c r="A56" s="26"/>
+      <c r="B56" s="20"/>
+      <c r="C56" s="22"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
       <c r="F56" s="3" t="s">
         <v>164</v>
       </c>
@@ -5494,36 +5581,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="A42:A43"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="E42:E43"/>
     <mergeCell ref="B54:H54"/>
     <mergeCell ref="A55:A56"/>
     <mergeCell ref="B55:B56"/>
     <mergeCell ref="C55:C56"/>
     <mergeCell ref="D55:D56"/>
     <mergeCell ref="E55:E56"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="A42:A43"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="B28:H28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?shared=false" xr:uid="{E4ADF2C1-50F1-4EB6-992B-DF51227C9B08}"/>
@@ -5633,26 +5720,26 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17" customHeight="1" thickBot="1">
       <c r="A1" s="12"/>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="21"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="13"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="27"/>
+      <c r="B2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="21" t="s">
         <v>162</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -5660,13 +5747,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" thickBot="1">
-      <c r="A3" s="14"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="18"/>
+      <c r="A3" s="28"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="22"/>
       <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="16"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="3" t="s">
         <v>4</v>
       </c>
@@ -5879,26 +5966,26 @@
     </row>
     <row r="16" spans="1:6" ht="17" thickBot="1">
       <c r="A16" s="12"/>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="21"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="16"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="13"/>
-      <c r="B17" s="15" t="s">
+      <c r="A17" s="27"/>
+      <c r="B17" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="21" t="s">
         <v>162</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F17" s="2" t="s">
@@ -5906,13 +5993,13 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="15" thickBot="1">
-      <c r="A18" s="14"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="18"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="22"/>
       <c r="D18" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="16"/>
+      <c r="E18" s="20"/>
       <c r="F18" s="3" t="s">
         <v>4</v>
       </c>
@@ -6107,26 +6194,26 @@
     </row>
     <row r="30" spans="1:6" ht="17" thickBot="1">
       <c r="A30" s="12"/>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="21"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="16"/>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="13"/>
-      <c r="B31" s="15" t="s">
+      <c r="A31" s="27"/>
+      <c r="B31" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="21" t="s">
         <v>162</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="15" t="s">
+      <c r="E31" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F31" s="2" t="s">
@@ -6134,13 +6221,13 @@
       </c>
     </row>
     <row r="32" spans="1:6" ht="15" thickBot="1">
-      <c r="A32" s="14"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="18"/>
+      <c r="A32" s="28"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="22"/>
       <c r="D32" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="16"/>
+      <c r="E32" s="20"/>
       <c r="F32" s="3" t="s">
         <v>4</v>
       </c>
@@ -6335,26 +6422,26 @@
     </row>
     <row r="44" spans="1:6" ht="17" thickBot="1">
       <c r="A44" s="12"/>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="20"/>
-      <c r="F44" s="21"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="16"/>
     </row>
     <row r="45" spans="1:6">
-      <c r="A45" s="13"/>
-      <c r="B45" s="15" t="s">
+      <c r="A45" s="27"/>
+      <c r="B45" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="17" t="s">
+      <c r="C45" s="21" t="s">
         <v>162</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="15" t="s">
+      <c r="E45" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F45" s="2" t="s">
@@ -6362,13 +6449,13 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="15" thickBot="1">
-      <c r="A46" s="14"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="18"/>
+      <c r="A46" s="28"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="22"/>
       <c r="D46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E46" s="16"/>
+      <c r="E46" s="20"/>
       <c r="F46" s="3" t="s">
         <v>4</v>
       </c>
@@ -6445,7 +6532,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="15" thickBot="1">
+    <row r="51" spans="1:6" ht="29.5" thickBot="1">
       <c r="A51" s="7"/>
       <c r="B51" s="6">
         <v>5</v>
@@ -6563,26 +6650,26 @@
     </row>
     <row r="58" spans="1:6" ht="17" thickBot="1">
       <c r="A58" s="12"/>
-      <c r="B58" s="19" t="s">
+      <c r="B58" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
-      <c r="E58" s="20"/>
-      <c r="F58" s="21"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15"/>
+      <c r="F58" s="16"/>
     </row>
     <row r="59" spans="1:6">
-      <c r="A59" s="13"/>
-      <c r="B59" s="15" t="s">
+      <c r="A59" s="27"/>
+      <c r="B59" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C59" s="17" t="s">
+      <c r="C59" s="21" t="s">
         <v>162</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E59" s="15" t="s">
+      <c r="E59" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F59" s="2" t="s">
@@ -6590,13 +6677,13 @@
       </c>
     </row>
     <row r="60" spans="1:6" ht="15" thickBot="1">
-      <c r="A60" s="14"/>
-      <c r="B60" s="16"/>
-      <c r="C60" s="18"/>
+      <c r="A60" s="28"/>
+      <c r="B60" s="20"/>
+      <c r="C60" s="22"/>
       <c r="D60" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E60" s="16"/>
+      <c r="E60" s="20"/>
       <c r="F60" s="3" t="s">
         <v>4</v>
       </c>
@@ -6791,26 +6878,26 @@
     </row>
     <row r="72" spans="1:6" ht="17" thickBot="1">
       <c r="A72" s="12"/>
-      <c r="B72" s="19" t="s">
+      <c r="B72" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="C72" s="20"/>
-      <c r="D72" s="20"/>
-      <c r="E72" s="20"/>
-      <c r="F72" s="21"/>
+      <c r="C72" s="15"/>
+      <c r="D72" s="15"/>
+      <c r="E72" s="15"/>
+      <c r="F72" s="16"/>
     </row>
     <row r="73" spans="1:6">
-      <c r="A73" s="13"/>
-      <c r="B73" s="15" t="s">
+      <c r="A73" s="27"/>
+      <c r="B73" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C73" s="17" t="s">
+      <c r="C73" s="21" t="s">
         <v>162</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E73" s="15" t="s">
+      <c r="E73" s="19" t="s">
         <v>5</v>
       </c>
       <c r="F73" s="2" t="s">
@@ -6818,13 +6905,13 @@
       </c>
     </row>
     <row r="74" spans="1:6" ht="15" thickBot="1">
-      <c r="A74" s="14"/>
-      <c r="B74" s="16"/>
-      <c r="C74" s="18"/>
+      <c r="A74" s="28"/>
+      <c r="B74" s="20"/>
+      <c r="C74" s="22"/>
       <c r="D74" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E74" s="16"/>
+      <c r="E74" s="20"/>
       <c r="F74" s="3" t="s">
         <v>4</v>
       </c>
@@ -7029,6 +7116,21 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A73:A74"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="B45:B46"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="B72:F72"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="A31:A32"/>
     <mergeCell ref="B31:B32"/>
@@ -7044,21 +7146,6 @@
     <mergeCell ref="C17:C18"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="B30:F30"/>
-    <mergeCell ref="A73:A74"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="B58:F58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="B72:F72"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" display="https://www.golfgenius.com/tournaments2/details/2232450552?round_index=&amp;player_stats_for_portal=true" xr:uid="{A3216F91-7A2C-4A18-8DDF-7BC507167619}"/>
@@ -7195,54 +7282,54 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:9" ht="17" customHeight="1" thickBot="1">
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="21"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="16"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" ht="15" thickBot="1">
-      <c r="A2" s="28"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="13"/>
+      <c r="B2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="19" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15" thickBot="1">
-      <c r="A3" s="28"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
     </row>
     <row r="4" spans="1:9" ht="58.5" thickBot="1">
       <c r="A4" s="5"/>
@@ -7418,55 +7505,55 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:9" ht="17" thickBot="1">
-      <c r="A11" s="28"/>
-      <c r="B11" s="19" t="s">
+      <c r="A11" s="13"/>
+      <c r="B11" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="21"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="16"/>
     </row>
     <row r="12" spans="1:9" ht="15" thickBot="1">
-      <c r="A12" s="28"/>
-      <c r="B12" s="15" t="s">
+      <c r="A12" s="13"/>
+      <c r="B12" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="G12" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="H12" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="19" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" thickBot="1">
-      <c r="A13" s="28"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
     </row>
     <row r="14" spans="1:9" ht="58.5" thickBot="1">
       <c r="A14" s="5"/>
@@ -7642,55 +7729,55 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="1:9" ht="17" thickBot="1">
-      <c r="A21" s="28"/>
-      <c r="B21" s="19" t="s">
+      <c r="A21" s="13"/>
+      <c r="B21" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="21"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="16"/>
     </row>
     <row r="22" spans="1:9" ht="15" thickBot="1">
-      <c r="A22" s="28"/>
-      <c r="B22" s="15" t="s">
+      <c r="A22" s="13"/>
+      <c r="B22" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="F22" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="H22" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="I22" s="15" t="s">
+      <c r="I22" s="19" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="15" thickBot="1">
-      <c r="A23" s="28"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
     </row>
     <row r="24" spans="1:9" ht="58.5" thickBot="1">
       <c r="A24" s="5"/>
@@ -7866,55 +7953,55 @@
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" ht="17" thickBot="1">
-      <c r="A31" s="28"/>
-      <c r="B31" s="19" t="s">
+      <c r="A31" s="13"/>
+      <c r="B31" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="21"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="16"/>
     </row>
     <row r="32" spans="1:9" ht="15" thickBot="1">
-      <c r="A32" s="28"/>
-      <c r="B32" s="15" t="s">
+      <c r="A32" s="13"/>
+      <c r="B32" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="C32" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="E32" s="15" t="s">
+      <c r="E32" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="F32" s="15" t="s">
+      <c r="F32" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="G32" s="15" t="s">
+      <c r="G32" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="H32" s="15" t="s">
+      <c r="H32" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="I32" s="15" t="s">
+      <c r="I32" s="19" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="15" thickBot="1">
-      <c r="A33" s="28"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
     </row>
     <row r="34" spans="1:9" ht="58.5" thickBot="1">
       <c r="A34" s="5"/>
@@ -8090,55 +8177,55 @@
       <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" ht="17" thickBot="1">
-      <c r="A41" s="28"/>
-      <c r="B41" s="19" t="s">
+      <c r="A41" s="13"/>
+      <c r="B41" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="20"/>
-      <c r="H41" s="20"/>
-      <c r="I41" s="21"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+      <c r="I41" s="16"/>
     </row>
     <row r="42" spans="1:9" ht="15" thickBot="1">
-      <c r="A42" s="28"/>
-      <c r="B42" s="15" t="s">
+      <c r="A42" s="13"/>
+      <c r="B42" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C42" s="17" t="s">
+      <c r="C42" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="E42" s="15" t="s">
+      <c r="E42" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="F42" s="15" t="s">
+      <c r="F42" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="G42" s="15" t="s">
+      <c r="G42" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="H42" s="15" t="s">
+      <c r="H42" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="I42" s="15" t="s">
+      <c r="I42" s="19" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="15" thickBot="1">
-      <c r="A43" s="28"/>
-      <c r="B43" s="16"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
-      <c r="F43" s="16"/>
-      <c r="G43" s="16"/>
-      <c r="H43" s="16"/>
-      <c r="I43" s="16"/>
+      <c r="A43" s="13"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="20"/>
     </row>
     <row r="44" spans="1:9" ht="73" thickBot="1">
       <c r="A44" s="5"/>
@@ -8314,55 +8401,55 @@
       <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" ht="17" thickBot="1">
-      <c r="A51" s="28"/>
-      <c r="B51" s="19" t="s">
+      <c r="A51" s="13"/>
+      <c r="B51" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="21"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+      <c r="H51" s="15"/>
+      <c r="I51" s="16"/>
     </row>
     <row r="52" spans="1:9" ht="15" thickBot="1">
-      <c r="A52" s="28"/>
-      <c r="B52" s="15" t="s">
+      <c r="A52" s="13"/>
+      <c r="B52" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C52" s="17" t="s">
+      <c r="C52" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="D52" s="15" t="s">
+      <c r="D52" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="E52" s="15" t="s">
+      <c r="E52" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="F52" s="15" t="s">
+      <c r="F52" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="G52" s="15" t="s">
+      <c r="G52" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="H52" s="15" t="s">
+      <c r="H52" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="I52" s="15" t="s">
+      <c r="I52" s="19" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="15" thickBot="1">
-      <c r="A53" s="28"/>
-      <c r="B53" s="16"/>
-      <c r="C53" s="18"/>
-      <c r="D53" s="16"/>
-      <c r="E53" s="16"/>
-      <c r="F53" s="16"/>
-      <c r="G53" s="16"/>
-      <c r="H53" s="16"/>
-      <c r="I53" s="16"/>
+      <c r="A53" s="13"/>
+      <c r="B53" s="20"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="20"/>
+      <c r="E53" s="20"/>
+      <c r="F53" s="20"/>
+      <c r="G53" s="20"/>
+      <c r="H53" s="20"/>
+      <c r="I53" s="20"/>
     </row>
     <row r="54" spans="1:9" ht="58.5" thickBot="1">
       <c r="A54" s="5"/>
@@ -8528,42 +8615,8 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="B51:I51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="H52:H53"/>
-    <mergeCell ref="I52:I53"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="F42:F43"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="H42:H43"/>
-    <mergeCell ref="I42:I43"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="G32:G33"/>
-    <mergeCell ref="H32:H33"/>
-    <mergeCell ref="I32:I33"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="B1:H1"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="B11:I11"/>
     <mergeCell ref="B12:B13"/>
@@ -8580,8 +8633,42 @@
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="H32:H33"/>
+    <mergeCell ref="I32:I33"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="H42:H43"/>
+    <mergeCell ref="I42:I43"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="G52:G53"/>
+    <mergeCell ref="H52:H53"/>
+    <mergeCell ref="I52:I53"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?shared=false" xr:uid="{97650E22-79F5-4347-9D75-ED6174696D39}"/>
@@ -8659,4 +8746,1911 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65E4259D-981B-4FFA-82AD-C6DBBFE41275}">
+  <dimension ref="A1:I74"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1" spans="1:9" ht="17" thickBot="1">
+      <c r="A1" s="30"/>
+      <c r="B1" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="38"/>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="31"/>
+      <c r="B2" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="32"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>279</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15" thickBot="1">
+      <c r="A4" s="33"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A5" s="5"/>
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="D5" s="4">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1</v>
+      </c>
+      <c r="G5" s="4">
+        <v>73</v>
+      </c>
+      <c r="H5" s="4">
+        <v>73</v>
+      </c>
+      <c r="I5" s="4">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A6" s="7"/>
+      <c r="B6" s="6">
+        <v>2</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="D6" s="6">
+        <v>3</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="6">
+        <v>3</v>
+      </c>
+      <c r="G6" s="6">
+        <v>72</v>
+      </c>
+      <c r="H6" s="6">
+        <v>75</v>
+      </c>
+      <c r="I6" s="6">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A7" s="5"/>
+      <c r="B7" s="4">
+        <v>3</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="D7" s="4">
+        <v>4</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4">
+        <v>2</v>
+      </c>
+      <c r="G7" s="4">
+        <v>74</v>
+      </c>
+      <c r="H7" s="4">
+        <v>74</v>
+      </c>
+      <c r="I7" s="4">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A8" s="7"/>
+      <c r="B8" s="6">
+        <v>4</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="D8" s="6">
+        <v>5</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6">
+        <v>76</v>
+      </c>
+      <c r="H8" s="6">
+        <v>73</v>
+      </c>
+      <c r="I8" s="6">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A9" s="5"/>
+      <c r="B9" s="4">
+        <v>5</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="D9" s="4">
+        <v>6</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="4">
+        <v>78</v>
+      </c>
+      <c r="H9" s="4">
+        <v>72</v>
+      </c>
+      <c r="I9" s="4">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A10" s="7"/>
+      <c r="B10" s="6">
+        <v>6</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="D10" s="6">
+        <v>9</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="6">
+        <v>6</v>
+      </c>
+      <c r="G10" s="6">
+        <v>75</v>
+      </c>
+      <c r="H10" s="6">
+        <v>78</v>
+      </c>
+      <c r="I10" s="6">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A11" s="5"/>
+      <c r="B11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="D11" s="4">
+        <v>10</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="4">
+        <v>7</v>
+      </c>
+      <c r="G11" s="4">
+        <v>75</v>
+      </c>
+      <c r="H11" s="4">
+        <v>79</v>
+      </c>
+      <c r="I11" s="4">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A12" s="7"/>
+      <c r="B12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="D12" s="6">
+        <v>10</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="6">
+        <v>8</v>
+      </c>
+      <c r="G12" s="6">
+        <v>74</v>
+      </c>
+      <c r="H12" s="6">
+        <v>80</v>
+      </c>
+      <c r="I12" s="6">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A13" s="5"/>
+      <c r="B13" s="4">
+        <v>9</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="D13" s="4">
+        <v>11</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="4">
+        <v>7</v>
+      </c>
+      <c r="G13" s="4">
+        <v>76</v>
+      </c>
+      <c r="H13" s="4">
+        <v>79</v>
+      </c>
+      <c r="I13" s="4">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A14" s="7"/>
+      <c r="B14" s="6">
+        <v>10</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="D14" s="6">
+        <v>18</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="6">
+        <v>8</v>
+      </c>
+      <c r="G14" s="6">
+        <v>82</v>
+      </c>
+      <c r="H14" s="6">
+        <v>80</v>
+      </c>
+      <c r="I14" s="6">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15" thickBot="1">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:9" ht="17" thickBot="1">
+      <c r="A16" s="30"/>
+      <c r="B16" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="16"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="31"/>
+      <c r="B17" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="H17" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="32"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>279</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15" thickBot="1">
+      <c r="A19" s="33"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A20" s="5"/>
+      <c r="B20" s="4">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="D20" s="4">
+        <v>-6</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" s="4">
+        <v>-4</v>
+      </c>
+      <c r="G20" s="4">
+        <v>70</v>
+      </c>
+      <c r="H20" s="4">
+        <v>68</v>
+      </c>
+      <c r="I20" s="4">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A21" s="7"/>
+      <c r="B21" s="6">
+        <v>2</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D21" s="6">
+        <v>-3</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="6">
+        <v>-1</v>
+      </c>
+      <c r="G21" s="6">
+        <v>70</v>
+      </c>
+      <c r="H21" s="6">
+        <v>71</v>
+      </c>
+      <c r="I21" s="6">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A22" s="5"/>
+      <c r="B22" s="4">
+        <v>3</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="D22" s="4">
+        <v>5</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" s="4">
+        <v>-3</v>
+      </c>
+      <c r="G22" s="4">
+        <v>80</v>
+      </c>
+      <c r="H22" s="4">
+        <v>69</v>
+      </c>
+      <c r="I22" s="4">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A23" s="7"/>
+      <c r="B23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="D23" s="6">
+        <v>8</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23" s="6">
+        <v>3</v>
+      </c>
+      <c r="G23" s="6">
+        <v>77</v>
+      </c>
+      <c r="H23" s="6">
+        <v>75</v>
+      </c>
+      <c r="I23" s="6">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A24" s="5"/>
+      <c r="B24" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="D24" s="4">
+        <v>8</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F24" s="4">
+        <v>7</v>
+      </c>
+      <c r="G24" s="4">
+        <v>73</v>
+      </c>
+      <c r="H24" s="4">
+        <v>79</v>
+      </c>
+      <c r="I24" s="4">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A25" s="7"/>
+      <c r="B25" s="6">
+        <v>6</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="D25" s="6">
+        <v>9</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" s="6">
+        <v>-2</v>
+      </c>
+      <c r="G25" s="6">
+        <v>83</v>
+      </c>
+      <c r="H25" s="6">
+        <v>70</v>
+      </c>
+      <c r="I25" s="6">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A26" s="5"/>
+      <c r="B26" s="4">
+        <v>7</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" s="4">
+        <v>12</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" s="4">
+        <v>8</v>
+      </c>
+      <c r="G26" s="4">
+        <v>76</v>
+      </c>
+      <c r="H26" s="4">
+        <v>80</v>
+      </c>
+      <c r="I26" s="4">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A27" s="7"/>
+      <c r="B27" s="6">
+        <v>8</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="D27" s="6">
+        <v>13</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F27" s="6">
+        <v>7</v>
+      </c>
+      <c r="G27" s="6">
+        <v>78</v>
+      </c>
+      <c r="H27" s="6">
+        <v>79</v>
+      </c>
+      <c r="I27" s="6">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A28" s="5"/>
+      <c r="B28" s="4">
+        <v>9</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="D28" s="4">
+        <v>16</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" s="4">
+        <v>9</v>
+      </c>
+      <c r="G28" s="4">
+        <v>79</v>
+      </c>
+      <c r="H28" s="4">
+        <v>81</v>
+      </c>
+      <c r="I28" s="4">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="44" thickBot="1">
+      <c r="A29" s="7"/>
+      <c r="B29" s="6">
+        <v>10</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D29" s="6">
+        <v>18</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" s="6">
+        <v>13</v>
+      </c>
+      <c r="G29" s="6">
+        <v>77</v>
+      </c>
+      <c r="H29" s="6">
+        <v>85</v>
+      </c>
+      <c r="I29" s="6">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15" thickBot="1">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+    </row>
+    <row r="31" spans="1:9" ht="17" thickBot="1">
+      <c r="A31" s="30"/>
+      <c r="B31" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="16"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="31"/>
+      <c r="B32" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="H32" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="32"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="35"/>
+      <c r="D33" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E33" s="29" t="s">
+        <v>279</v>
+      </c>
+      <c r="F33" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
+      <c r="I33" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15" thickBot="1">
+      <c r="A34" s="33"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="3"/>
+    </row>
+    <row r="35" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A35" s="5"/>
+      <c r="B35" s="4">
+        <v>1</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="D35" s="4">
+        <v>-3</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G35" s="4">
+        <v>69</v>
+      </c>
+      <c r="H35" s="4">
+        <v>72</v>
+      </c>
+      <c r="I35" s="4">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A36" s="7"/>
+      <c r="B36" s="6">
+        <v>2</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="D36" s="6">
+        <v>1</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F36" s="6">
+        <v>2</v>
+      </c>
+      <c r="G36" s="6">
+        <v>71</v>
+      </c>
+      <c r="H36" s="6">
+        <v>74</v>
+      </c>
+      <c r="I36" s="6">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A37" s="5"/>
+      <c r="B37" s="4">
+        <v>3</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D37" s="4">
+        <v>5</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F37" s="4">
+        <v>1</v>
+      </c>
+      <c r="G37" s="4">
+        <v>76</v>
+      </c>
+      <c r="H37" s="4">
+        <v>73</v>
+      </c>
+      <c r="I37" s="4">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="44" thickBot="1">
+      <c r="A38" s="7"/>
+      <c r="B38" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="D38" s="6">
+        <v>7</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F38" s="6">
+        <v>3</v>
+      </c>
+      <c r="G38" s="6">
+        <v>76</v>
+      </c>
+      <c r="H38" s="6">
+        <v>75</v>
+      </c>
+      <c r="I38" s="6">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A39" s="5"/>
+      <c r="B39" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="D39" s="4">
+        <v>7</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F39" s="4">
+        <v>7</v>
+      </c>
+      <c r="G39" s="4">
+        <v>72</v>
+      </c>
+      <c r="H39" s="4">
+        <v>79</v>
+      </c>
+      <c r="I39" s="4">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A40" s="7"/>
+      <c r="B40" s="6">
+        <v>6</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="D40" s="6">
+        <v>8</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" s="6">
+        <v>1</v>
+      </c>
+      <c r="G40" s="6">
+        <v>79</v>
+      </c>
+      <c r="H40" s="6">
+        <v>73</v>
+      </c>
+      <c r="I40" s="6">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A41" s="5"/>
+      <c r="B41" s="4">
+        <v>7</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D41" s="4">
+        <v>12</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" s="4">
+        <v>3</v>
+      </c>
+      <c r="G41" s="4">
+        <v>81</v>
+      </c>
+      <c r="H41" s="4">
+        <v>75</v>
+      </c>
+      <c r="I41" s="4">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A42" s="7"/>
+      <c r="B42" s="6">
+        <v>8</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="D42" s="6">
+        <v>13</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" s="6">
+        <v>7</v>
+      </c>
+      <c r="G42" s="6">
+        <v>78</v>
+      </c>
+      <c r="H42" s="6">
+        <v>79</v>
+      </c>
+      <c r="I42" s="6">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A43" s="5"/>
+      <c r="B43" s="4">
+        <v>9</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="D43" s="4">
+        <v>14</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" s="4">
+        <v>7</v>
+      </c>
+      <c r="G43" s="4">
+        <v>79</v>
+      </c>
+      <c r="H43" s="4">
+        <v>79</v>
+      </c>
+      <c r="I43" s="4">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A44" s="7"/>
+      <c r="B44" s="6">
+        <v>10</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D44" s="6">
+        <v>25</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F44" s="6">
+        <v>10</v>
+      </c>
+      <c r="G44" s="6">
+        <v>87</v>
+      </c>
+      <c r="H44" s="6">
+        <v>82</v>
+      </c>
+      <c r="I44" s="6">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15" thickBot="1">
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+    </row>
+    <row r="46" spans="1:9" ht="17" thickBot="1">
+      <c r="A46" s="30"/>
+      <c r="B46" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="I46" s="16"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="31"/>
+      <c r="B47" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G47" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="H47" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="32"/>
+      <c r="B48" s="34"/>
+      <c r="C48" s="35"/>
+      <c r="D48" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E48" s="29" t="s">
+        <v>279</v>
+      </c>
+      <c r="F48" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G48" s="34"/>
+      <c r="H48" s="34"/>
+      <c r="I48" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="15" thickBot="1">
+      <c r="A49" s="33"/>
+      <c r="B49" s="20"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G49" s="20"/>
+      <c r="H49" s="20"/>
+      <c r="I49" s="3"/>
+    </row>
+    <row r="50" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A50" s="5"/>
+      <c r="B50" s="4">
+        <v>1</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F50" s="4">
+        <v>-2</v>
+      </c>
+      <c r="G50" s="4">
+        <v>74</v>
+      </c>
+      <c r="H50" s="4">
+        <v>70</v>
+      </c>
+      <c r="I50" s="4">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A51" s="7"/>
+      <c r="B51" s="6">
+        <v>2</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="D51" s="6">
+        <v>2</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F51" s="6">
+        <v>5</v>
+      </c>
+      <c r="G51" s="6">
+        <v>69</v>
+      </c>
+      <c r="H51" s="6">
+        <v>77</v>
+      </c>
+      <c r="I51" s="6">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A52" s="5"/>
+      <c r="B52" s="4">
+        <v>3</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D52" s="4">
+        <v>9</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F52" s="4">
+        <v>1</v>
+      </c>
+      <c r="G52" s="4">
+        <v>80</v>
+      </c>
+      <c r="H52" s="4">
+        <v>73</v>
+      </c>
+      <c r="I52" s="4">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A53" s="7"/>
+      <c r="B53" s="6">
+        <v>4</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="D53" s="6">
+        <v>10</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F53" s="6">
+        <v>7</v>
+      </c>
+      <c r="G53" s="6">
+        <v>75</v>
+      </c>
+      <c r="H53" s="6">
+        <v>79</v>
+      </c>
+      <c r="I53" s="6">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A54" s="5"/>
+      <c r="B54" s="4">
+        <v>5</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="D54" s="4">
+        <v>12</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F54" s="4">
+        <v>11</v>
+      </c>
+      <c r="G54" s="4">
+        <v>73</v>
+      </c>
+      <c r="H54" s="4">
+        <v>83</v>
+      </c>
+      <c r="I54" s="4">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A55" s="7"/>
+      <c r="B55" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="D55" s="6">
+        <v>15</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F55" s="6">
+        <v>8</v>
+      </c>
+      <c r="G55" s="6">
+        <v>79</v>
+      </c>
+      <c r="H55" s="6">
+        <v>80</v>
+      </c>
+      <c r="I55" s="6">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A56" s="5"/>
+      <c r="B56" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="D56" s="4">
+        <v>15</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F56" s="4">
+        <v>6</v>
+      </c>
+      <c r="G56" s="4">
+        <v>81</v>
+      </c>
+      <c r="H56" s="4">
+        <v>78</v>
+      </c>
+      <c r="I56" s="4">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A57" s="7"/>
+      <c r="B57" s="6">
+        <v>8</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="D57" s="6">
+        <v>20</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F57" s="6">
+        <v>9</v>
+      </c>
+      <c r="G57" s="6">
+        <v>83</v>
+      </c>
+      <c r="H57" s="6">
+        <v>81</v>
+      </c>
+      <c r="I57" s="6">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A58" s="5"/>
+      <c r="B58" s="4">
+        <v>9</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="D58" s="4">
+        <v>25</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F58" s="4">
+        <v>15</v>
+      </c>
+      <c r="G58" s="4">
+        <v>82</v>
+      </c>
+      <c r="H58" s="4">
+        <v>87</v>
+      </c>
+      <c r="I58" s="4">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A59" s="7"/>
+      <c r="B59" s="6">
+        <v>10</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D59" s="6">
+        <v>28</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" s="6">
+        <v>18</v>
+      </c>
+      <c r="G59" s="6">
+        <v>82</v>
+      </c>
+      <c r="H59" s="6">
+        <v>90</v>
+      </c>
+      <c r="I59" s="6">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="15" thickBot="1">
+      <c r="A60" s="1"/>
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
+    </row>
+    <row r="61" spans="1:9" ht="17" thickBot="1">
+      <c r="A61" s="30"/>
+      <c r="B61" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="15"/>
+      <c r="I61" s="16"/>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" s="31"/>
+      <c r="B62" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G62" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="H62" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="A63" s="32"/>
+      <c r="B63" s="34"/>
+      <c r="C63" s="35"/>
+      <c r="D63" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E63" s="29" t="s">
+        <v>279</v>
+      </c>
+      <c r="F63" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G63" s="34"/>
+      <c r="H63" s="34"/>
+      <c r="I63" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="15" thickBot="1">
+      <c r="A64" s="33"/>
+      <c r="B64" s="20"/>
+      <c r="C64" s="22"/>
+      <c r="D64" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="G64" s="20"/>
+      <c r="H64" s="20"/>
+      <c r="I64" s="3"/>
+    </row>
+    <row r="65" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A65" s="5"/>
+      <c r="B65" s="4">
+        <v>1</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="D65" s="4">
+        <v>1</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F65" s="4">
+        <v>-2</v>
+      </c>
+      <c r="G65" s="4">
+        <v>75</v>
+      </c>
+      <c r="H65" s="4">
+        <v>70</v>
+      </c>
+      <c r="I65" s="4">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A66" s="7"/>
+      <c r="B66" s="6">
+        <v>2</v>
+      </c>
+      <c r="C66" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D66" s="6">
+        <v>5</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F66" s="6">
+        <v>5</v>
+      </c>
+      <c r="G66" s="6">
+        <v>72</v>
+      </c>
+      <c r="H66" s="6">
+        <v>77</v>
+      </c>
+      <c r="I66" s="6">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A67" s="5"/>
+      <c r="B67" s="4">
+        <v>3</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="D67" s="4">
+        <v>6</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G67" s="4">
+        <v>78</v>
+      </c>
+      <c r="H67" s="4">
+        <v>72</v>
+      </c>
+      <c r="I67" s="4">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A68" s="7"/>
+      <c r="B68" s="6">
+        <v>4</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D68" s="6">
+        <v>8</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F68" s="6">
+        <v>6</v>
+      </c>
+      <c r="G68" s="6">
+        <v>74</v>
+      </c>
+      <c r="H68" s="6">
+        <v>78</v>
+      </c>
+      <c r="I68" s="6">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A69" s="5"/>
+      <c r="B69" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="D69" s="4">
+        <v>10</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69" s="4">
+        <v>8</v>
+      </c>
+      <c r="G69" s="4">
+        <v>74</v>
+      </c>
+      <c r="H69" s="4">
+        <v>80</v>
+      </c>
+      <c r="I69" s="4">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A70" s="7"/>
+      <c r="B70" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C70" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D70" s="6">
+        <v>10</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F70" s="6">
+        <v>10</v>
+      </c>
+      <c r="G70" s="6">
+        <v>72</v>
+      </c>
+      <c r="H70" s="6">
+        <v>82</v>
+      </c>
+      <c r="I70" s="6">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A71" s="5"/>
+      <c r="B71" s="4">
+        <v>7</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="D71" s="4">
+        <v>13</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F71" s="4">
+        <v>7</v>
+      </c>
+      <c r="G71" s="4">
+        <v>78</v>
+      </c>
+      <c r="H71" s="4">
+        <v>79</v>
+      </c>
+      <c r="I71" s="4">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A72" s="7"/>
+      <c r="B72" s="6">
+        <v>8</v>
+      </c>
+      <c r="C72" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="D72" s="6">
+        <v>15</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F72" s="6">
+        <v>9</v>
+      </c>
+      <c r="G72" s="6">
+        <v>78</v>
+      </c>
+      <c r="H72" s="6">
+        <v>81</v>
+      </c>
+      <c r="I72" s="6">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A73" s="5"/>
+      <c r="B73" s="4">
+        <v>9</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="D73" s="4">
+        <v>34</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F73" s="4">
+        <v>-1</v>
+      </c>
+      <c r="G73" s="4">
+        <v>107</v>
+      </c>
+      <c r="H73" s="4">
+        <v>71</v>
+      </c>
+      <c r="I73" s="4">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="29.5" thickBot="1">
+      <c r="A74" s="7"/>
+      <c r="B74" s="6">
+        <v>10</v>
+      </c>
+      <c r="C74" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="D74" s="6">
+        <v>61</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F74" s="6">
+        <v>29</v>
+      </c>
+      <c r="G74" s="6">
+        <v>104</v>
+      </c>
+      <c r="H74" s="6">
+        <v>101</v>
+      </c>
+      <c r="I74" s="6">
+        <v>205</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="B61:I61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="B62:B64"/>
+    <mergeCell ref="C62:C64"/>
+    <mergeCell ref="G62:G64"/>
+    <mergeCell ref="H62:H64"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="G47:G49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="G17:G19"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="G2:G4"/>
+    <mergeCell ref="H2:H4"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A5" r:id="rId1" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{CADF7DEE-B18A-45CB-9E77-D35C2DE06EAE}"/>
+    <hyperlink ref="C5" r:id="rId2" display="https://www.golfgenius.com/tournaments2/details/2344000549?round_index=&amp;player_stats_for_portal=true" xr:uid="{3398A9DC-28A5-4454-928D-F981E3FEF4C4}"/>
+    <hyperlink ref="A6" r:id="rId3" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{48D7943A-D594-4886-9AD9-DD1D589A4AC9}"/>
+    <hyperlink ref="C6" r:id="rId4" display="https://www.golfgenius.com/tournaments2/details/2344000568?round_index=&amp;player_stats_for_portal=true" xr:uid="{A87F4618-544C-4B0A-AB78-0F60A17F8EAE}"/>
+    <hyperlink ref="A7" r:id="rId5" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{4D01AF15-36E6-4EF9-BD6F-CF26B2B41C7D}"/>
+    <hyperlink ref="C7" r:id="rId6" display="https://www.golfgenius.com/tournaments2/details/2344000532?round_index=&amp;player_stats_for_portal=true" xr:uid="{942F88D8-2996-4242-8965-62186634236C}"/>
+    <hyperlink ref="A8" r:id="rId7" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{7AF701A6-E8E4-4D0C-B293-FC7A4DE3271D}"/>
+    <hyperlink ref="C8" r:id="rId8" display="https://www.golfgenius.com/tournaments2/details/2344000551?round_index=&amp;player_stats_for_portal=true" xr:uid="{A46FBEF7-59DC-4052-8BDC-748FB5D3344F}"/>
+    <hyperlink ref="A9" r:id="rId9" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{1193CF08-9848-4DBF-B07E-704F4715574A}"/>
+    <hyperlink ref="C9" r:id="rId10" display="https://www.golfgenius.com/tournaments2/details/2344000565?round_index=&amp;player_stats_for_portal=true" xr:uid="{7D694BAE-9E93-4D6E-8CD3-22932F53DC4D}"/>
+    <hyperlink ref="A10" r:id="rId11" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{5668E744-EEB4-437E-95AB-453AA7C34E36}"/>
+    <hyperlink ref="C10" r:id="rId12" display="https://www.golfgenius.com/tournaments2/details/2344000567?round_index=&amp;player_stats_for_portal=true" xr:uid="{3AEE4594-0CC3-4011-8A2F-E52C432C53FD}"/>
+    <hyperlink ref="A11" r:id="rId13" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{380CCD3D-BC73-4677-8A82-D86A5290563A}"/>
+    <hyperlink ref="C11" r:id="rId14" display="https://www.golfgenius.com/tournaments2/details/2344000548?round_index=&amp;player_stats_for_portal=true" xr:uid="{CC8CB35B-CD47-4C49-BF54-DA25A5FDC333}"/>
+    <hyperlink ref="A12" r:id="rId15" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{0ACBDDCC-2B84-45C4-BE65-B465994DE4B9}"/>
+    <hyperlink ref="C12" r:id="rId16" display="https://www.golfgenius.com/tournaments2/details/2344000550?round_index=&amp;player_stats_for_portal=true" xr:uid="{F2C987E8-AB29-48B4-9020-607542BF990C}"/>
+    <hyperlink ref="A13" r:id="rId17" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{42906911-B5B4-4F82-B35D-9D6B68DBA656}"/>
+    <hyperlink ref="C13" r:id="rId18" display="https://www.golfgenius.com/tournaments2/details/2344000566?round_index=&amp;player_stats_for_portal=true" xr:uid="{27D7B0D0-96F6-4084-A06F-B5A55569CF3F}"/>
+    <hyperlink ref="A14" r:id="rId19" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{4DA6D509-DCD5-4F84-BD43-36FA7E8A46CA}"/>
+    <hyperlink ref="C14" r:id="rId20" display="https://www.golfgenius.com/tournaments2/details/2344000533?round_index=&amp;player_stats_for_portal=true" xr:uid="{081F19A8-9835-4AD0-9308-5B130E30E6FF}"/>
+    <hyperlink ref="A20" r:id="rId21" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{F1D08EEC-6A86-427F-B24C-4D03036BA7F4}"/>
+    <hyperlink ref="C20" r:id="rId22" display="https://www.golfgenius.com/tournaments2/details/2344000536?round_index=&amp;player_stats_for_portal=true" xr:uid="{0B046D8A-A5DC-47B2-89D7-CC372798E164}"/>
+    <hyperlink ref="A21" r:id="rId23" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{ECC010C8-9DF7-43D5-9DA6-F2000FA8DC65}"/>
+    <hyperlink ref="C21" r:id="rId24" display="https://www.golfgenius.com/tournaments2/details/2344000535?round_index=&amp;player_stats_for_portal=true" xr:uid="{B60FC92C-95A9-432B-905B-A3BF82D1DA66}"/>
+    <hyperlink ref="A22" r:id="rId25" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{69CCE66B-5611-4815-BFC5-1CCE09097E16}"/>
+    <hyperlink ref="C22" r:id="rId26" display="https://www.golfgenius.com/tournaments2/details/2344000572?round_index=&amp;player_stats_for_portal=true" xr:uid="{4E3C3162-4AE5-46E4-BF94-0E430EA2F2F5}"/>
+    <hyperlink ref="A23" r:id="rId27" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{C952BD84-BAE1-4526-B4C6-E94E78494598}"/>
+    <hyperlink ref="C23" r:id="rId28" display="https://www.golfgenius.com/tournaments2/details/2344000571?round_index=&amp;player_stats_for_portal=true" xr:uid="{72E1B1D9-ADDF-4EC1-82AA-5760A8C06074}"/>
+    <hyperlink ref="A24" r:id="rId29" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{927C24C8-D2A4-45FA-A157-EB7782A1947A}"/>
+    <hyperlink ref="C24" r:id="rId30" display="https://www.golfgenius.com/tournaments2/details/2344000552?round_index=&amp;player_stats_for_portal=true" xr:uid="{A3863F7E-E5E8-45CE-A15E-E9BCF69B0779}"/>
+    <hyperlink ref="A25" r:id="rId31" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{407C2896-0BBC-4C86-AA50-3B02A3C1351F}"/>
+    <hyperlink ref="C25" r:id="rId32" display="https://www.golfgenius.com/tournaments2/details/2344000553?round_index=&amp;player_stats_for_portal=true" xr:uid="{02188C54-0BBD-4BB4-930C-3AF5616BC135}"/>
+    <hyperlink ref="A26" r:id="rId33" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{9DAFA46A-EE0E-41E8-AB9C-44FB5C60A03B}"/>
+    <hyperlink ref="C26" r:id="rId34" display="https://www.golfgenius.com/tournaments2/details/2344000570?round_index=&amp;player_stats_for_portal=true" xr:uid="{5464BDCD-7FFA-4CEC-BDDE-97DC1F894C2B}"/>
+    <hyperlink ref="A27" r:id="rId35" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{A836B657-36DB-4659-B56F-D943E8B38CAE}"/>
+    <hyperlink ref="C27" r:id="rId36" display="https://www.golfgenius.com/tournaments2/details/2344000534?round_index=&amp;player_stats_for_portal=true" xr:uid="{2F46972A-AF26-495C-B373-CB7874EACF55}"/>
+    <hyperlink ref="A28" r:id="rId37" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{4160F1B2-2AE6-4181-8F5A-34328E767D5B}"/>
+    <hyperlink ref="C28" r:id="rId38" display="https://www.golfgenius.com/tournaments2/details/2344000569?round_index=&amp;player_stats_for_portal=true" xr:uid="{8A50DB04-B5EE-4B59-8CC3-56163A0AF924}"/>
+    <hyperlink ref="A29" r:id="rId39" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{D99BB468-D59F-4718-8FCE-0069BE957BBB}"/>
+    <hyperlink ref="C29" r:id="rId40" display="https://www.golfgenius.com/tournaments2/details/2344000554?round_index=&amp;player_stats_for_portal=true" xr:uid="{BC03411B-C992-432A-B0CC-82C55EFDDB71}"/>
+    <hyperlink ref="A35" r:id="rId41" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{D4689AF4-3CB1-42E4-9B1A-B7D19021AC95}"/>
+    <hyperlink ref="C35" r:id="rId42" display="https://www.golfgenius.com/tournaments2/details/2344000539?round_index=&amp;player_stats_for_portal=true" xr:uid="{C407B6B6-D3CA-49A7-96D4-6253C0C4C8BC}"/>
+    <hyperlink ref="A36" r:id="rId43" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{D04489C8-FC8E-4768-AE00-A3B4BBC454F3}"/>
+    <hyperlink ref="C36" r:id="rId44" display="https://www.golfgenius.com/tournaments2/details/2344000575?round_index=&amp;player_stats_for_portal=true" xr:uid="{3E32BF4F-C17D-41F3-9532-18EA06295157}"/>
+    <hyperlink ref="A37" r:id="rId45" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{DC9D732E-35DE-4A7E-9FB1-22C0CA0B5ACC}"/>
+    <hyperlink ref="C37" r:id="rId46" display="https://www.golfgenius.com/tournaments2/details/2344000540?round_index=&amp;player_stats_for_portal=true" xr:uid="{D6C9F9FB-DD49-4C8A-9FAE-C0BC68D7E7FA}"/>
+    <hyperlink ref="A38" r:id="rId47" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{D78312F2-07C5-48D1-B236-F5DB3ED3E607}"/>
+    <hyperlink ref="C38" r:id="rId48" display="https://www.golfgenius.com/tournaments2/details/2344000538?round_index=&amp;player_stats_for_portal=true" xr:uid="{B99BC9C3-AC6D-42CC-A8F9-E0E1FF88EE5B}"/>
+    <hyperlink ref="A39" r:id="rId49" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{7E195761-22BD-4330-A046-C947EFE51C13}"/>
+    <hyperlink ref="C39" r:id="rId50" display="https://www.golfgenius.com/tournaments2/details/2344000537?round_index=&amp;player_stats_for_portal=true" xr:uid="{2E238214-B009-445D-B806-F7B8B3334B0C}"/>
+    <hyperlink ref="A40" r:id="rId51" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{E0967793-79A6-48DA-8993-731EF2F51A11}"/>
+    <hyperlink ref="C40" r:id="rId52" display="https://www.golfgenius.com/tournaments2/details/2344000555?round_index=&amp;player_stats_for_portal=true" xr:uid="{78A2D3C9-CBE2-4475-81D0-BF43D3DC84B8}"/>
+    <hyperlink ref="A41" r:id="rId53" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{A20D6673-44F7-4B28-A7B6-3C11B9CA0080}"/>
+    <hyperlink ref="C41" r:id="rId54" display="https://www.golfgenius.com/tournaments2/details/2344000556?round_index=&amp;player_stats_for_portal=true" xr:uid="{C4E22097-1194-458C-BADC-CAC33FD2A8AE}"/>
+    <hyperlink ref="A42" r:id="rId55" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{1424C338-E215-4CBA-9DC7-0C7BB6109C18}"/>
+    <hyperlink ref="C42" r:id="rId56" display="https://www.golfgenius.com/tournaments2/details/2344000557?round_index=&amp;player_stats_for_portal=true" xr:uid="{6AA2DD9F-F596-40B9-951B-9A4E2C14CF4A}"/>
+    <hyperlink ref="A43" r:id="rId57" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{B424BE0E-EDD2-48C8-B6C2-D69A0A95736D}"/>
+    <hyperlink ref="C43" r:id="rId58" display="https://www.golfgenius.com/tournaments2/details/2344000558?round_index=&amp;player_stats_for_portal=true" xr:uid="{992BE01A-5450-445A-A05B-DCEB7F85545B}"/>
+    <hyperlink ref="A44" r:id="rId59" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{F3D866E0-C67F-4DB4-AEEB-B3B7AF334084}"/>
+    <hyperlink ref="C44" r:id="rId60" display="https://www.golfgenius.com/tournaments2/details/2344000574?round_index=&amp;player_stats_for_portal=true" xr:uid="{9DA0151B-A98C-46EC-AB8E-F4C608C820F0}"/>
+    <hyperlink ref="A50" r:id="rId61" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{E01E2AF2-ED78-45D7-9FC8-487EC0596067}"/>
+    <hyperlink ref="C50" r:id="rId62" display="https://www.golfgenius.com/tournaments2/details/2344000559?round_index=&amp;player_stats_for_portal=true" xr:uid="{69E400BB-932F-4B05-8A4D-279B51AB975C}"/>
+    <hyperlink ref="A51" r:id="rId63" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{A0C7096C-270D-4DE4-B2DA-D13993B238E9}"/>
+    <hyperlink ref="C51" r:id="rId64" display="https://www.golfgenius.com/tournaments2/details/2344000581?round_index=&amp;player_stats_for_portal=true" xr:uid="{A4A03851-CBFE-486D-98BD-6D476EA801A3}"/>
+    <hyperlink ref="A52" r:id="rId65" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{8C208439-5EF4-4435-9F61-EC30BD832AB6}"/>
+    <hyperlink ref="C52" r:id="rId66" display="https://www.golfgenius.com/tournaments2/details/2344000542?round_index=&amp;player_stats_for_portal=true" xr:uid="{8F122FCE-9A87-4F00-92E6-B4F05A3F765B}"/>
+    <hyperlink ref="A53" r:id="rId67" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{1E0E29F2-3363-43F4-ABFD-807130AD7367}"/>
+    <hyperlink ref="C53" r:id="rId68" display="https://www.golfgenius.com/tournaments2/details/2344000573?round_index=&amp;player_stats_for_portal=true" xr:uid="{339B5854-6789-46E0-83A9-C326AE9A9FAE}"/>
+    <hyperlink ref="A54" r:id="rId69" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{0887CB0B-6D81-4D6C-85DC-79F0BCE9DDEB}"/>
+    <hyperlink ref="C54" r:id="rId70" display="https://www.golfgenius.com/tournaments2/details/2344000564?round_index=&amp;player_stats_for_portal=true" xr:uid="{DB798912-F356-4D02-A346-07FB2E102079}"/>
+    <hyperlink ref="A55" r:id="rId71" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{B5548DDE-5F4F-404C-A8C1-2837CD6E9E32}"/>
+    <hyperlink ref="C55" r:id="rId72" display="https://www.golfgenius.com/tournaments2/details/2344000561?round_index=&amp;player_stats_for_portal=true" xr:uid="{E9775AF7-F971-4934-A894-F84F210C8C52}"/>
+    <hyperlink ref="A56" r:id="rId73" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{B83F886D-22FB-4932-8313-A8A9DC7C3D5C}"/>
+    <hyperlink ref="C56" r:id="rId74" display="https://www.golfgenius.com/tournaments2/details/2344000543?round_index=&amp;player_stats_for_portal=true" xr:uid="{118854C1-478D-44EF-9629-614FCBD0604E}"/>
+    <hyperlink ref="A57" r:id="rId75" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{9DC5014C-35CE-4ECB-B770-CF6D032D8293}"/>
+    <hyperlink ref="C57" r:id="rId76" display="https://www.golfgenius.com/tournaments2/details/2344000578?round_index=&amp;player_stats_for_portal=true" xr:uid="{2289E3EC-540A-4921-BF0B-C4161F9C3162}"/>
+    <hyperlink ref="A58" r:id="rId77" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{C0254BAB-3F3A-46BD-A322-68566765A9A6}"/>
+    <hyperlink ref="C58" r:id="rId78" display="https://www.golfgenius.com/tournaments2/details/2344000576?round_index=&amp;player_stats_for_portal=true" xr:uid="{D9C2DEA9-B938-453F-92B7-27DFE9870F90}"/>
+    <hyperlink ref="A59" r:id="rId79" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{6264BADE-E0F3-419C-9DCB-CACB8D3ED38F}"/>
+    <hyperlink ref="C59" r:id="rId80" display="https://www.golfgenius.com/tournaments2/details/2344000541?round_index=&amp;player_stats_for_portal=true" xr:uid="{B441775D-9A5B-4F0F-BA4A-47F170F4C2D4}"/>
+    <hyperlink ref="A65" r:id="rId81" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{74A285B4-28DD-47A4-B4DA-B778F25E7114}"/>
+    <hyperlink ref="C65" r:id="rId82" display="https://www.golfgenius.com/tournaments2/details/2344000547?round_index=&amp;player_stats_for_portal=true" xr:uid="{6B953DE6-47DF-4B5C-A7B3-C916780B2F43}"/>
+    <hyperlink ref="A66" r:id="rId83" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{835411D2-B2DC-4CF1-85DF-3FA33792A4B9}"/>
+    <hyperlink ref="C66" r:id="rId84" display="https://www.golfgenius.com/tournaments2/details/2344000580?round_index=&amp;player_stats_for_portal=true" xr:uid="{4AD01A55-7632-4414-A5B8-C8992E8F9049}"/>
+    <hyperlink ref="A67" r:id="rId85" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{9ACFC2B4-0073-40B6-8716-4735A8F69BBB}"/>
+    <hyperlink ref="C67" r:id="rId86" display="https://www.golfgenius.com/tournaments2/details/2344000579?round_index=&amp;player_stats_for_portal=true" xr:uid="{53E6BBDF-2B99-4FCA-ADB5-70E07C1A90EF}"/>
+    <hyperlink ref="A68" r:id="rId87" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{FBFAAEAA-6B64-4F72-9FC8-23866EB3E20D}"/>
+    <hyperlink ref="C68" r:id="rId88" display="https://www.golfgenius.com/tournaments2/details/2344000546?round_index=&amp;player_stats_for_portal=true" xr:uid="{D347A1E9-9399-4517-8125-0141BCFFC2C3}"/>
+    <hyperlink ref="A69" r:id="rId89" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{43636270-1C9D-40AE-A45F-10572EA99527}"/>
+    <hyperlink ref="C69" r:id="rId90" display="https://www.golfgenius.com/tournaments2/details/2344000544?round_index=&amp;player_stats_for_portal=true" xr:uid="{8F73F03B-89ED-4D9D-B156-0DD45117785A}"/>
+    <hyperlink ref="A70" r:id="rId91" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{57509AE8-A970-44D5-94C2-40B2BA742376}"/>
+    <hyperlink ref="C70" r:id="rId92" display="https://www.golfgenius.com/tournaments2/details/2344000562?round_index=&amp;player_stats_for_portal=true" xr:uid="{183E16FD-F38C-408E-8122-8A5B452ECA92}"/>
+    <hyperlink ref="A71" r:id="rId93" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{806580EB-506A-42C1-8D62-5697358AD269}"/>
+    <hyperlink ref="C71" r:id="rId94" display="https://www.golfgenius.com/tournaments2/details/2344000577?round_index=&amp;player_stats_for_portal=true" xr:uid="{C729D8B2-F36B-4C54-AC3C-962F31CB0C97}"/>
+    <hyperlink ref="A72" r:id="rId95" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{AF990601-2D0C-4694-8FA3-7026CCEB4C43}"/>
+    <hyperlink ref="C72" r:id="rId96" display="https://www.golfgenius.com/tournaments2/details/2344000560?round_index=&amp;player_stats_for_portal=true" xr:uid="{9E0D495F-ECE4-4AE1-8F02-F1F5104FF63F}"/>
+    <hyperlink ref="A73" r:id="rId97" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{574A9221-6BDE-411E-A76F-E4F7C3053CC9}"/>
+    <hyperlink ref="C73" r:id="rId98" display="https://www.golfgenius.com/tournaments2/details/2344000545?round_index=&amp;player_stats_for_portal=true" xr:uid="{21B1E04B-07A8-4084-96F9-EA1C78CA6C31}"/>
+    <hyperlink ref="A74" r:id="rId99" display="https://www.golfgenius.com/leagues/492667/widgets/tournament_results?round=1682939&amp;shared=false" xr:uid="{4CEB3776-2C4F-4214-8649-913638ED4C46}"/>
+    <hyperlink ref="C74" r:id="rId100" display="https://www.golfgenius.com/tournaments2/details/2344000563?round_index=&amp;player_stats_for_portal=true" xr:uid="{06929661-D3FB-481F-A565-715878AC9F79}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>